<commit_message>
docs: add quantum computing hardware and fault tolerance papers
</commit_message>
<xml_diff>
--- a/metadata/QComputing.xlsx
+++ b/metadata/QComputing.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R31f945d75e5d4d36"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Ra2780099a1ad4bc3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -376,19 +376,19 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>A Review on Models and Applications of Quantum Computing</x:v>
+        <x:v>Benchmarking fault-tolerant quantum computing hardware via QLOPS</x:v>
       </x:c>
       <x:c r="B4" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>ACM</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>Eduard Grigoryan; Sachin Kumar; Placido Rogério Pinheiro</x:v>
+        <x:v>Linghang Kong; Fang Zhang; Jianxin Chen</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>https://doi.org/10.3390/quantum7030039</x:v>
+        <x:v>https://doi.org/10.1145/3797968</x:v>
       </x:c>
       <x:c r="F4" t="str">
         <x:v>QComputing</x:v>
@@ -396,19 +396,19 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Quantum computing: foundations, algorithms, and emerging applications</x:v>
+        <x:v>Low-overhead fault-tolerant quantum computation by gauging logical operators</x:v>
       </x:c>
       <x:c r="B5" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Frontiers</x:v>
+        <x:v>Nature Physics</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>V. Raseena</x:v>
+        <x:v>Dominic J. Williamson; Theodore J. Yoder</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>https://doi.org/10.3389/frqst.2025.1723319</x:v>
+        <x:v>https://doi.org/10.1038/s41567-026-03220-8</x:v>
       </x:c>
       <x:c r="F5" t="str">
         <x:v>QComputing</x:v>
@@ -416,19 +416,19 @@
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Quantum Computing: Foundations, Architecture and Applications</x:v>
+        <x:v>Improved quantum processor logical error rates via correction and detection</x:v>
       </x:c>
       <x:c r="B6" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Wiley</x:v>
+        <x:v>Nature</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>Christopher Columbus Chinnappan; Palani Thanaraj Krishnan; Elakiya Elamaran; Rajakumar Arul; T. Sunil Kumar</x:v>
+        <x:v>A. Paetznick et al.</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>https://doi.org/10.1002/eng2.70337</x:v>
+        <x:v>https://doi.org/10.1038/s41586-026-10628-y</x:v>
       </x:c>
       <x:c r="F6" t="str">
         <x:v>QComputing</x:v>
@@ -436,19 +436,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>A survey on quantum computing: Transforming cryptography, AI/ML, blockchain, and network communication</x:v>
+        <x:v>A Review on Models and Applications of Quantum Computing</x:v>
       </x:c>
       <x:c r="B7" t="n">
         <x:v>2025</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Elsevier</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Shruti Kundu; Twinkle Gupta; Akash Sardar; Anjan Bandyopadhyay; Sujata Swain; Saurav Mallik</x:v>
+        <x:v>Eduard Grigoryan; Sachin Kumar; Placido Rogério Pinheiro</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>https://doi.org/10.1016/j.fraope.2025.100371</x:v>
+        <x:v>https://doi.org/10.3390/quantum7030039</x:v>
       </x:c>
       <x:c r="F7" t="str">
         <x:v>QComputing</x:v>
@@ -456,19 +456,19 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>Quantum computing with Qiskit</x:v>
+        <x:v>Quantum computing: foundations, algorithms, and emerging applications</x:v>
       </x:c>
       <x:c r="B8" t="n">
-        <x:v>2024</x:v>
+        <x:v>2025</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>Frontiers</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>Javadi-Abhari, Ali, et al.</x:v>
+        <x:v>V. Raseena</x:v>
       </x:c>
       <x:c r="E8" t="str">
-        <x:v>https://arxiv.org/abs/2405.08810</x:v>
+        <x:v>https://doi.org/10.3389/frqst.2025.1723319</x:v>
       </x:c>
       <x:c r="F8" t="str">
         <x:v>QComputing</x:v>
@@ -476,140 +476,140 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
+        <x:v>Quantum Computing: Foundations, Architecture and Applications</x:v>
+      </x:c>
+      <x:c r="B9" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>Wiley</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Christopher Columbus Chinnappan; Palani Thanaraj Krishnan; Elakiya Elamaran; Rajakumar Arul; T. Sunil Kumar</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>https://doi.org/10.1002/eng2.70337</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>A survey on quantum computing: Transforming cryptography, AI/ML, blockchain, and network communication</x:v>
+      </x:c>
+      <x:c r="B10" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Elsevier</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>Shruti Kundu; Twinkle Gupta; Akash Sardar; Anjan Bandyopadhyay; Sujata Swain; Saurav Mallik</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>https://doi.org/10.1016/j.fraope.2025.100371</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>Distributed quantum computing across an optical network link</x:v>
+      </x:c>
+      <x:c r="B11" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>Nature</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>D. Main; P. Drmota; D. P. Nadlinger; E. M. Ainley; A. Agrawal; B. C. Nichol; R. Srinivas; G. Araneda; D. M. Lucas</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>https://doi.org/10.1038/s41586-024-08404-x</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>An 11-qubit atom processor in silicon</x:v>
+      </x:c>
+      <x:c r="B12" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C12" t="str">
+        <x:v>Nature</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>Hermann Edlbauer et al.</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>https://doi.org/10.1038/s41586-025-09827-w</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>Hardware-efficient quantum error correction via concatenated bosonic qubits</x:v>
+      </x:c>
+      <x:c r="B13" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C13" t="str">
+        <x:v>Nature</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>Harald Putterman et al.</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>https://doi.org/10.1038/s41586-025-08642-7</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>Quantum computing with Qiskit</x:v>
+      </x:c>
+      <x:c r="B14" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>arXiv</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>Javadi-Abhari, Ali, et al.</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>https://arxiv.org/abs/2405.08810</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
         <x:v>Quantum Computing and AI in the Cloud
 </x:v>
       </x:c>
-      <x:c r="B9" t="n">
+      <x:c r="B15" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C9" t="str">
+      <x:c r="C15" t="str">
         <x:v>Journal of Computational Intelligence and Robotics</x:v>
       </x:c>
-      <x:c r="D9" t="str">
+      <x:c r="D15" t="str">
         <x:v>Padmanaban, Harish.</x:v>
       </x:c>
-      <x:c r="E9" t="str">
+      <x:c r="E15" t="str">
         <x:v>https://thesciencebrigade.com/jcir/article/view/116</x:v>
-      </x:c>
-      <x:c r="F9" t="str">
-        <x:v>QComputing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
-      <x:c r="A10" t="str">
-        <x:v>Quantum Machine Learning: Exploring the Potential of Quantum Computing forAI Applications</x:v>
-      </x:c>
-      <x:c r="B10" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C10" t="str">
-        <x:v>Artificial Intelligence General Science (JAIGS)</x:v>
-      </x:c>
-      <x:c r="D10" t="str">
-        <x:v>Potter, Kaledio, and Dylan Stilinski.</x:v>
-      </x:c>
-      <x:c r="E10" t="str">
-        <x:v>https://easychair.org/publications/preprint/bb78/download</x:v>
-      </x:c>
-      <x:c r="F10" t="str">
-        <x:v>QComputing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11">
-      <x:c r="A11" t="str">
-        <x:v>Quantum Computing and Artificial Intelligence: Synergies and Challenges</x:v>
-      </x:c>
-      <x:c r="B11" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C11" t="str">
-        <x:v>Journal of Artificial Intelligence General science (JAIGS)</x:v>
-      </x:c>
-      <x:c r="D11" t="str">
-        <x:v>Shuford, Jeff.</x:v>
-      </x:c>
-      <x:c r="E11" t="str">
-        <x:v>https://ojs.boulibrary.com/index.php/JAIGS/article/view/35</x:v>
-      </x:c>
-      <x:c r="F11" t="str">
-        <x:v>QComputing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12">
-      <x:c r="A12" t="str">
-        <x:v>LEVERAGING QUANTUM COMPUTING FOR INCLUSIVE AND RESPONSIBLE AI DEVELOPMENT: A CONCEPTUAL AND REVIEW FRAMEWORK</x:v>
-      </x:c>
-      <x:c r="B12" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C12" t="str">
-        <x:v>Computer Science &amp; IT Research Journal </x:v>
-      </x:c>
-      <x:c r="D12" t="str">
-        <x:v>Olorunsogo, Temidayo, Boma Sonimiteim Jacks, and Olakunle Abayomi Ajala.</x:v>
-      </x:c>
-      <x:c r="E12" t="str">
-        <x:v>https://fepbl.com/index.php/csitrj/article/view/927</x:v>
-      </x:c>
-      <x:c r="F12" t="str">
-        <x:v>QComputing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13">
-      <x:c r="A13" t="str">
-        <x:v>Quantum Intelligence: Merging AI and Quantum Computing for Unprecedented Power.</x:v>
-      </x:c>
-      <x:c r="B13" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C13" t="str">
-        <x:v>International Conference on Trends in Quantum Computing and Emerging Business Technologies</x:v>
-      </x:c>
-      <x:c r="D13" t="str">
-        <x:v>Kumar, Sonu, Simran Simran, and Manjit Singh.</x:v>
-      </x:c>
-      <x:c r="E13" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10545163</x:v>
-      </x:c>
-      <x:c r="F13" t="str">
-        <x:v>QComputing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14">
-      <x:c r="A14" t="str">
-        <x:v>Quantum computing applications for Internet of Things</x:v>
-      </x:c>
-      <x:c r="B14" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C14" t="str">
-        <x:v>IET Quantum Communication </x:v>
-      </x:c>
-      <x:c r="D14" t="str">
-        <x:v>Peelam, Mritunjay Shall, Anjaney Asreet Rout, and Vinay Chamola.</x:v>
-      </x:c>
-      <x:c r="E14" t="str">
-        <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/full/10.1049/qtc2.12079</x:v>
-      </x:c>
-      <x:c r="F14" t="str">
-        <x:v>QComputing</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
-        <x:v>Quantum autoencoders for communication-efficient cloud computing</x:v>
-      </x:c>
-      <x:c r="B15" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C15" t="str">
-        <x:v>Springer</x:v>
-      </x:c>
-      <x:c r="D15" t="str">
-        <x:v>Yan Zhu, Ge Bai, Yuexuan Wang, Tongyang Li &amp; Giulio Chiribella</x:v>
-      </x:c>
-      <x:c r="E15" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00112-5</x:v>
       </x:c>
       <x:c r="F15" t="str">
         <x:v>QComputing</x:v>
@@ -617,19 +617,19 @@
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>Quantum computing for a profusion of postman problem variants</x:v>
+        <x:v>Quantum Machine Learning: Exploring the Potential of Quantum Computing forAI Applications</x:v>
       </x:c>
       <x:c r="B16" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C16" t="str">
-        <x:v>Springer</x:v>
+        <x:v>Artificial Intelligence General Science (JAIGS)</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>Joel E. Pion, Christian F. A. Negre &amp; Susan M. Mniszewski</x:v>
+        <x:v>Potter, Kaledio, and Dylan Stilinski.</x:v>
       </x:c>
       <x:c r="E16" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00111-6</x:v>
+        <x:v>https://easychair.org/publications/preprint/bb78/download</x:v>
       </x:c>
       <x:c r="F16" t="str">
         <x:v>QComputing</x:v>
@@ -637,19 +637,19 @@
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>Faster quantum state decomposition with Tucker tensor approximation</x:v>
+        <x:v>Quantum Computing and Artificial Intelligence: Synergies and Challenges</x:v>
       </x:c>
       <x:c r="B17" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C17" t="str">
-        <x:v>Springer</x:v>
+        <x:v>Journal of Artificial Intelligence General science (JAIGS)</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>Protasov Stanislav &amp; Lisnichenko Marina </x:v>
+        <x:v>Shuford, Jeff.</x:v>
       </x:c>
       <x:c r="E17" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00113-4</x:v>
+        <x:v>https://ojs.boulibrary.com/index.php/JAIGS/article/view/35</x:v>
       </x:c>
       <x:c r="F17" t="str">
         <x:v>QComputing</x:v>
@@ -657,19 +657,19 @@
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>The quantum threat to blockchain: summary and timeline analysis</x:v>
+        <x:v>LEVERAGING QUANTUM COMPUTING FOR INCLUSIVE AND RESPONSIBLE AI DEVELOPMENT: A CONCEPTUAL AND REVIEW FRAMEWORK</x:v>
       </x:c>
       <x:c r="B18" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C18" t="str">
-        <x:v>Springer</x:v>
+        <x:v>Computer Science &amp; IT Research Journal </x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>Kai Schärer &amp; Marco Comuzzi</x:v>
+        <x:v>Olorunsogo, Temidayo, Boma Sonimiteim Jacks, and Olakunle Abayomi Ajala.</x:v>
       </x:c>
       <x:c r="E18" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00105-4</x:v>
+        <x:v>https://fepbl.com/index.php/csitrj/article/view/927</x:v>
       </x:c>
       <x:c r="F18" t="str">
         <x:v>QComputing</x:v>
@@ -677,19 +677,19 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>The quantum realization of image linear gray enhancement</x:v>
+        <x:v>Quantum Intelligence: Merging AI and Quantum Computing for Unprecedented Power.</x:v>
       </x:c>
       <x:c r="B19" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>Springer</x:v>
+        <x:v>International Conference on Trends in Quantum Computing and Emerging Business Technologies</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>Kai Liu, Yuxing Wei &amp; Hai-Sheng Li</x:v>
+        <x:v>Kumar, Sonu, Simran Simran, and Manjit Singh.</x:v>
       </x:c>
       <x:c r="E19" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00102-7</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10545163</x:v>
       </x:c>
       <x:c r="F19" t="str">
         <x:v>QComputing</x:v>
@@ -697,19 +697,19 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>Quantum computing for near-term applications in generative chemistry and drug discovery</x:v>
+        <x:v>Quantum computing applications for Internet of Things</x:v>
       </x:c>
       <x:c r="B20" t="n">
-        <x:v>2023</x:v>
+        <x:v>2024</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>IET Quantum Communication </x:v>
       </x:c>
       <x:c r="D20" t="str">
-        <x:v>Alexey Pyrkov, Alex Aliper, Dmitry Bezrukov, Yen-Chu Lin, Daniil Polykovskiy, Petrina Kamya, Feng Ren, Alex Zhavoronkov </x:v>
+        <x:v>Peelam, Mritunjay Shall, Anjaney Asreet Rout, and Vinay Chamola.</x:v>
       </x:c>
       <x:c r="E20" t="str">
-        <x:v>https://doi.org/10.1016/j.drudis.2023.103675</x:v>
+        <x:v>https://ietresearch.onlinelibrary.wiley.com/doi/full/10.1049/qtc2.12079</x:v>
       </x:c>
       <x:c r="F20" t="str">
         <x:v>QComputing</x:v>
@@ -717,19 +717,19 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
-        <x:v>The state of quantum computing applications in health and medicine</x:v>
+        <x:v>Quantum autoencoders for communication-efficient cloud computing</x:v>
       </x:c>
       <x:c r="B21" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>Cambridge Core</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D21" t="str">
-        <x:v>Frederik F. Flöther</x:v>
+        <x:v>Yan Zhu, Ge Bai, Yuexuan Wang, Tongyang Li &amp; Giulio Chiribella</x:v>
       </x:c>
       <x:c r="E21" t="str">
-        <x:v>https://doi.org/10.1017/qut.2023.4</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00112-5</x:v>
       </x:c>
       <x:c r="F21" t="str">
         <x:v>QComputing</x:v>
@@ -737,41 +737,167 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>Business Renaissance: Opportunities and Challenges at the Dawn of the Quantum Computing Era</x:v>
+        <x:v>Quantum computing for a profusion of postman problem variants</x:v>
       </x:c>
       <x:c r="B22" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C22" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>Joel E. Pion, Christian F. A. Negre &amp; Susan M. Mniszewski</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>https://doi.org/10.1007/s42484-023-00111-6</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" t="str">
+        <x:v>Faster quantum state decomposition with Tucker tensor approximation</x:v>
+      </x:c>
+      <x:c r="B23" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C23" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D23" t="str">
+        <x:v>Protasov Stanislav &amp; Lisnichenko Marina </x:v>
+      </x:c>
+      <x:c r="E23" t="str">
+        <x:v>https://doi.org/10.1007/s42484-023-00113-4</x:v>
+      </x:c>
+      <x:c r="F23" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" t="str">
+        <x:v>The quantum threat to blockchain: summary and timeline analysis</x:v>
+      </x:c>
+      <x:c r="B24" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C24" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D24" t="str">
+        <x:v>Kai Schärer &amp; Marco Comuzzi</x:v>
+      </x:c>
+      <x:c r="E24" t="str">
+        <x:v>https://doi.org/10.1007/s42484-023-00105-4</x:v>
+      </x:c>
+      <x:c r="F24" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" t="str">
+        <x:v>The quantum realization of image linear gray enhancement</x:v>
+      </x:c>
+      <x:c r="B25" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C25" t="str">
+        <x:v>Springer</x:v>
+      </x:c>
+      <x:c r="D25" t="str">
+        <x:v>Kai Liu, Yuxing Wei &amp; Hai-Sheng Li</x:v>
+      </x:c>
+      <x:c r="E25" t="str">
+        <x:v>https://doi.org/10.1007/s42484-023-00102-7</x:v>
+      </x:c>
+      <x:c r="F25" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>Quantum computing for near-term applications in generative chemistry and drug discovery</x:v>
+      </x:c>
+      <x:c r="B26" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>ScienceDirect</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>Alexey Pyrkov, Alex Aliper, Dmitry Bezrukov, Yen-Chu Lin, Daniil Polykovskiy, Petrina Kamya, Feng Ren, Alex Zhavoronkov </x:v>
+      </x:c>
+      <x:c r="E26" t="str">
+        <x:v>https://doi.org/10.1016/j.drudis.2023.103675</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" t="str">
+        <x:v>The state of quantum computing applications in health and medicine</x:v>
+      </x:c>
+      <x:c r="B27" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C27" t="str">
+        <x:v>Cambridge Core</x:v>
+      </x:c>
+      <x:c r="D27" t="str">
+        <x:v>Frederik F. Flöther</x:v>
+      </x:c>
+      <x:c r="E27" t="str">
+        <x:v>https://doi.org/10.1017/qut.2023.4</x:v>
+      </x:c>
+      <x:c r="F27" t="str">
+        <x:v>QComputing</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" t="str">
+        <x:v>Business Renaissance: Opportunities and Challenges at the Dawn of the Quantum Computing Era</x:v>
+      </x:c>
+      <x:c r="B28" t="n">
+        <x:v>2023</x:v>
+      </x:c>
+      <x:c r="C28" t="str">
         <x:v>MDPI</x:v>
       </x:c>
-      <x:c r="D22" t="str">
+      <x:c r="D28" t="str">
         <x:v> Meng-Leong How, Sin-Mei Cheah</x:v>
       </x:c>
-      <x:c r="E22" t="str">
+      <x:c r="E28" t="str">
         <x:v>https://doi.org/10.3390/businesses3040036</x:v>
       </x:c>
-      <x:c r="F22" t="str">
+      <x:c r="F28" t="str">
         <x:v>QComputing</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="Rcfa6a85671e34a01"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R4cefff4a708e4258"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="R5de1dc6cc2684f57"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R4c297b7358c64062"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="Rb4194bb87a1b4606"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R1ef25a111c7c4970"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="Rbb99a7f0a8c24ada"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="R734fdf83ed61443a"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R6ca0947e35a341c9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R8de6034b9ebc4fff"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="R841140bad6a0467b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="R7c666c5e1d73401c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R39a7db2baa1c4365"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="Rdd970d94740b47d0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="R15e16b209cf8489f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R13b91824ae954d6c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="R7b6058f5977e4a01"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="R842071a5d1c349fa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="R44414febcc2d4431"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="R04ec3437c8864de7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="R29bbd13219fc43e5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="Re8beb591ba8942da"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="Rac8bf2aeb7214ce4"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="R1bf30fabbf8347b5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="R7a57324d78d349b0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="Ra5ec5f4a74524fb5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="Re35b6714c4dc4bfc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="R179a5cc4410b41b1"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R5e2392487e8c4aac"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="Rdc0260e3cfec4bd7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="Rbc220a5ff42d4963"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="Ra3833aeae9794917"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="Rdff9811229e54332"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R6fbdb598813a4793"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="R1ec4b89542d54a11"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="Ref14694d127e4cdb"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>